<commit_message>
Polish admin UI, merge Home+Dashboard, add employee data management
- Refresh visual design (Noto Sans KR font, gradient KPI cards, nav
  icons, avatar badge, softer shadows) across the sidebar admin shell
- Merge Home and Dashboard into a single "홈" page at the top of the
  nav; /dashboard now redirects there for backward compatibility
- Rename "가상 GHD 판단 기준" nav label to "관련 내규"
- Add proper HTML pages for 직원 데이터 and 관련 내규 (previously
  raw JSON test routes) via new -view routes
- Add employee data entry: manual form + Excel bulk upload, both
  writing through employee_service (Supabase or local Excel) and
  invalidating the cache so Home/Proactive Care reflect it immediately
- Adjust two demo employees' start_date/employment_period so Proactive
  Care shows a realistic HIGH/MEDIUM/LOW severity mix instead of only
  LOW

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/employees.xlsx
+++ b/data/employees.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="직원명단" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="직원명단" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'직원명단'!$A$3:$I$33</definedName>
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -84,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -93,6 +95,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -554,14 +559,12 @@
           <t>생산직(조립)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>2021-09-04</t>
-        </is>
+      <c r="F4" s="4" t="n">
+        <v>45928</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>2년</t>
+          <t>1년</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -601,14 +604,12 @@
           <t>통번역 지원</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>2024-02-08</t>
-        </is>
+      <c r="F5" s="4" t="n">
+        <v>45777</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>1년</t>
+          <t>1년 6개월</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">

</xml_diff>